<commit_message>
Excel Reading operations are completed
</commit_message>
<xml_diff>
--- a/src/main/java/com/test/resources/testJavaExcel.xlsx
+++ b/src/main/java/com/test/resources/testJavaExcel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Divya\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7dee5f4522bdc06d/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE78517-0F03-4BB3-AC7C-7311DF5E485D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{0EE78517-0F03-4BB3-AC7C-7311DF5E485D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E91CBE71-F165-4179-8459-58454C8EF3C4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>country</t>
   </si>
@@ -131,6 +131,12 @@
   </si>
   <si>
     <t>maki@789</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>admin123</t>
   </si>
 </sst>
 </file>
@@ -612,7 +618,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F09FA25-C4E4-41E0-8FBD-1BD6CB9AD00D}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -651,6 +657,14 @@
         <v>34</v>
       </c>
     </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{4F42BC09-A898-48B5-8155-4EB01B7F2A04}"/>

</xml_diff>

<commit_message>
Excel write operations added
</commit_message>
<xml_diff>
--- a/src/main/java/com/test/resources/testJavaExcel.xlsx
+++ b/src/main/java/com/test/resources/testJavaExcel.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7dee5f4522bdc06d/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7dee5f4522bdc06d/Desktop/selenium_data_driven_framework/src/main/java/com/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{0EE78517-0F03-4BB3-AC7C-7311DF5E485D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E91CBE71-F165-4179-8459-58454C8EF3C4}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{0EE78517-0F03-4BB3-AC7C-7311DF5E485D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EC99869-8659-4CAE-8F36-57179A2B769F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
   <si>
     <t>country</t>
   </si>
@@ -121,12 +121,6 @@
     <t>baki@123</t>
   </si>
   <si>
-    <t>suki456</t>
-  </si>
-  <si>
-    <t>suki@456</t>
-  </si>
-  <si>
     <t>maki789</t>
   </si>
   <si>
@@ -137,12 +131,31 @@
   </si>
   <si>
     <t>admin123</t>
+  </si>
+  <si>
+    <t>ramu</t>
+  </si>
+  <si>
+    <t>ramandh</t>
+  </si>
+  <si>
+    <t>standard_user</t>
+  </si>
+  <si>
+    <t>secret_sauce</t>
+  </si>
+  <si>
+    <t>fail</t>
+  </si>
+  <si>
+    <t>Pass</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -200,6 +213,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -469,145 +486,145 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="0">
         <v>500000</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="0">
         <v>800000</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="0">
         <v>3200000</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="0">
         <v>2300000</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="A6" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="0">
         <v>7400000</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="0">
         <v>2200000</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="0">
         <v>430000</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" t="s" s="0">
         <v>21</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="0">
         <v>630000</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="0">
         <v>6900000</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="A11" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="0">
         <v>5400000</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="A12" t="s" s="0">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="0">
         <v>1200000</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="A13" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="0">
         <v>6400000</v>
       </c>
     </row>
@@ -618,58 +635,80 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F09FA25-C4E4-41E0-8FBD-1BD6CB9AD00D}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="14.6640625"/>
+    <col min="2" max="2" customWidth="true" width="15.5546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>28</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>29</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>30</v>
       </c>
+      <c r="C2" t="s" s="0">
+        <v>39</v>
+      </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>31</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>32</v>
       </c>
+      <c r="C3" t="s" s="0">
+        <v>39</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
         <v>33</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s" s="0">
         <v>34</v>
       </c>
+      <c r="C4" t="s" s="0">
+        <v>39</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" t="s" s="0">
         <v>35</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" t="s" s="0">
         <v>36</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{4F42BC09-A898-48B5-8155-4EB01B7F2A04}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{866479B2-53A5-46C5-9540-495167BE7BC2}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{31C47F5A-ED58-4EE6-9BA1-484B188C8E37}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{31C47F5A-ED58-4EE6-9BA1-484B188C8E37}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>